<commit_message>
train model to extract causal
</commit_message>
<xml_diff>
--- a/configs/causal_triggers.xlsx
+++ b/configs/causal_triggers.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C32"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -898,6 +898,66 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>56</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>nhờ</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>57</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>góp phần</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>58</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>thúc đẩy</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>pos</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>59</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>do</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>neu</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>